<commit_message>
mejorando la parte de productos
</commit_message>
<xml_diff>
--- a/Documents/caapd-facturacion/escritorio/Base de datos/PADRON_MES_2026-09.xlsx
+++ b/Documents/caapd-facturacion/escritorio/Base de datos/PADRON_MES_2026-09.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15 00:42:21</t>
+          <t>2026-10-15 02:33:48</t>
         </is>
       </c>
     </row>
@@ -1418,11 +1418,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="P8" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+      <c r="P8" s="11" t="inlineStr"/>
       <c r="Q8" s="14" t="inlineStr">
         <is>
           <t>30778043</t>
@@ -1852,7 +1848,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="P5" s="11" t="inlineStr"/>
+      <c r="P5" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="Q5" s="14" t="inlineStr">
         <is>
           <t>30769321</t>
@@ -2942,11 +2942,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="P9" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+      <c r="P9" s="11" t="inlineStr"/>
       <c r="Q9" s="14" t="inlineStr">
         <is>
           <t>75849301</t>

</xml_diff>

<commit_message>
Ultima version hasta ahora
</commit_message>
<xml_diff>
--- a/Documents/caapd-facturacion/escritorio/Base de datos/PADRON_MES_2026-09.xlsx
+++ b/Documents/caapd-facturacion/escritorio/Base de datos/PADRON_MES_2026-09.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15 01:35:28</t>
+          <t>2026-10-15 04:35:01</t>
         </is>
       </c>
     </row>
@@ -6706,6 +6706,50 @@
           "precio_m3": 4.0
         }
       ]
+    },
+    "B": {
+      "nombre": "Comercial",
+      "cargo_fijo": 2.5,
+      "tarifa_desague": 0.0,
+      "rangos": [
+        {
+          "m3_desde": 0,
+          "m3_hasta": 10,
+          "precio_m3": 1.5
+        },
+        {
+          "m3_desde": 10,
+          "m3_hasta": 20,
+          "precio_m3": 2.0
+        },
+        {
+          "m3_desde": 20,
+          "m3_hasta": null,
+          "precio_m3": 3.0
+        }
+      ]
+    },
+    "C": {
+      "nombre": "Estatal / Social",
+      "cargo_fijo": 1.5,
+      "tarifa_desague": 0.0,
+      "rangos": [
+        {
+          "m3_desde": 0,
+          "m3_hasta": 10,
+          "precio_m3": 1.0
+        },
+        {
+          "m3_desde": 10,
+          "m3_hasta": 20,
+          "precio_m3": 1.5
+        },
+        {
+          "m3_desde": 20,
+          "m3_hasta": null,
+          "precio_m3": 2.5
+        }
+      ]
     }
   },
   "lectores": {

</xml_diff>